<commit_message>
Remove NO_D from feasible DAC location -> too far away
</commit_message>
<xml_diff>
--- a/dac_offshore/clean_data/technologies_new/NewTechnologies.xlsx
+++ b/dac_offshore/clean_data/technologies_new/NewTechnologies.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwiegner\PycharmProjects\AdOpT_DAC-Offshore\dac_offshore\clean_data\technologies_new\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7C7090-4892-42A5-AFF8-9ADD71AFF5B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D24750F-34C7-4616-9712-703932F086BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{64A87C74-33CB-4EAC-BDF2-6E9087B161C6}"/>
+    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="11260" xr2:uid="{64A87C74-33CB-4EAC-BDF2-6E9087B161C6}"/>
   </bookViews>
   <sheets>
     <sheet name="NewTechnologies" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">NewTechnologies!$A$1:$E$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">NewTechnologies!$A$1:$F$56</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="106">
   <si>
     <t>offshore_new</t>
   </si>
@@ -352,6 +352,12 @@
   </si>
   <si>
     <t>co2storage</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Too far away for DAC</t>
   </si>
 </sst>
 </file>
@@ -711,15 +717,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E56"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F56"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="25.85546875" customWidth="1"/>
+    <col min="2" max="2" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="25.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -735,8 +741,11 @@
       <c r="E1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>93</v>
       </c>
@@ -747,7 +756,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>95</v>
       </c>
@@ -758,7 +767,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>94</v>
       </c>
@@ -769,7 +778,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>61</v>
       </c>
@@ -783,7 +792,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>60</v>
       </c>
@@ -797,7 +806,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>59</v>
       </c>
@@ -811,7 +820,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>58</v>
       </c>
@@ -825,7 +834,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>57</v>
       </c>
@@ -839,7 +848,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>56</v>
       </c>
@@ -853,7 +862,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>55</v>
       </c>
@@ -867,7 +876,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -881,7 +890,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>53</v>
       </c>
@@ -895,7 +904,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>52</v>
       </c>
@@ -905,11 +914,11 @@
       <c r="C14" t="s">
         <v>64</v>
       </c>
-      <c r="E14" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>51</v>
       </c>
@@ -923,7 +932,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>50</v>
       </c>
@@ -937,7 +946,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -951,7 +960,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -965,7 +974,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -976,7 +985,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -987,7 +996,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -998,7 +1007,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -1009,7 +1018,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -1020,7 +1029,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -1031,7 +1040,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -1042,7 +1051,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>26</v>
       </c>
@@ -1056,7 +1065,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -1067,7 +1076,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>37</v>
       </c>
@@ -1081,7 +1090,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>38</v>
       </c>
@@ -1095,7 +1104,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>39</v>
       </c>
@@ -1109,7 +1118,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>6</v>
       </c>
@@ -1123,7 +1132,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>10</v>
       </c>
@@ -1137,7 +1146,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -1151,7 +1160,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>20</v>
       </c>
@@ -1165,7 +1174,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -1179,7 +1188,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>24</v>
       </c>
@@ -1193,7 +1202,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>33</v>
       </c>
@@ -1207,7 +1216,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>34</v>
       </c>
@@ -1221,7 +1230,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>35</v>
       </c>
@@ -1235,7 +1244,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>36</v>
       </c>
@@ -1249,7 +1258,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -1263,7 +1272,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>9</v>
       </c>
@@ -1277,7 +1286,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>16</v>
       </c>
@@ -1291,7 +1300,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>17</v>
       </c>
@@ -1305,7 +1314,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>18</v>
       </c>
@@ -1319,7 +1328,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>19</v>
       </c>
@@ -1333,7 +1342,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -1347,7 +1356,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>28</v>
       </c>
@@ -1361,7 +1370,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>29</v>
       </c>
@@ -1375,7 +1384,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>30</v>
       </c>
@@ -1389,7 +1398,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>31</v>
       </c>
@@ -1403,7 +1412,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>32</v>
       </c>
@@ -1417,7 +1426,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>40</v>
       </c>
@@ -1431,7 +1440,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>41</v>
       </c>
@@ -1445,7 +1454,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>42</v>
       </c>
@@ -1459,7 +1468,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>43</v>
       </c>
@@ -1474,11 +1483,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E38" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E56">
-      <sortCondition ref="B1:B38"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:F56" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="3"/>
@@ -1492,13 +1497,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4641E15-13AD-4645-88BC-55D8D2E876ED}">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>63</v>
       </c>
@@ -1510,7 +1515,7 @@
         <v>'RE_only': 'RE only',</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>70</v>
       </c>
@@ -1522,7 +1527,7 @@
         <v>'Battery_on': 'Battery (onshore only)',</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -1534,7 +1539,7 @@
         <v>'Battery_off': 'Battery (offshore only)',</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1546,7 +1551,7 @@
         <v>'Battery_all': 'Battery (all)',</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>45</v>
       </c>
@@ -1558,7 +1563,7 @@
         <v>'ElectricityGrid_all': 'Grid Expansion (all)',</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>46</v>
       </c>
@@ -1570,7 +1575,7 @@
         <v>'Hydrogen_Baseline': 'Hydrogen (all)',</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>72</v>
       </c>
@@ -1582,7 +1587,7 @@
         <v>'Hydrogen_H1': 'Hydrogen (no storage)',</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>73</v>
       </c>
@@ -1594,7 +1599,7 @@
         <v>'Hydrogen_H2': 'Hydrogen (no hydrogen offshore)',</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>74</v>
       </c>
@@ -1606,7 +1611,7 @@
         <v>'Hydrogen_H3': 'Hydrogen (no hydrogen onshore)',</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>75</v>
       </c>
@@ -1618,7 +1623,7 @@
         <v>'Hydrogen_H4': 'Hydrogen (local use only)',</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>47</v>
       </c>
@@ -1630,7 +1635,7 @@
         <v>'All': 'All Pathways',</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>66</v>
       </c>
@@ -1643,7 +1648,7 @@
         <v>'RE_only_no_onshore_wind': 'RE only - no onshore wind',</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>76</v>
       </c>
@@ -1656,7 +1661,7 @@
         <v>'Battery_on_no_onshore_wind': 'Battery (onshore only) - no onshore wind',</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -1669,7 +1674,7 @@
         <v>'Battery_off_no_onshore_wind': 'Battery (offshore only) - no onshore wind',</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -1682,7 +1687,7 @@
         <v>'Battery_all_no_onshore_wind': 'Battery (all) - no onshore wind',</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>68</v>
       </c>
@@ -1695,7 +1700,7 @@
         <v>'ElectricityGrid_all_no_onshore_wind': 'Grid Expansion (all) - no onshore wind',</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>69</v>
       </c>
@@ -1708,7 +1713,7 @@
         <v>'Hydrogen_Baseline_no_onshore_wind': 'Hydrogen (all) - no onshore wind',</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>78</v>
       </c>
@@ -1721,7 +1726,7 @@
         <v>'Hydrogen_H1_no_onshore_wind': 'Hydrogen (no storage) - no onshore wind',</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>79</v>
       </c>
@@ -1734,7 +1739,7 @@
         <v>'Hydrogen_H2_no_onshore_wind': 'Hydrogen (no hydrogen offshore) - no onshore wind',</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>80</v>
       </c>
@@ -1747,7 +1752,7 @@
         <v>'Hydrogen_H3_no_onshore_wind': 'Hydrogen (no hydrogen onshore) - no onshore wind',</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>81</v>
       </c>
@@ -1760,7 +1765,7 @@
         <v>'Hydrogen_H4_no_onshore_wind': 'Hydrogen (local use only) - no onshore wind',</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>65</v>
       </c>

</xml_diff>

<commit_message>
Updated NewTechnologies.xlsx to remove duplicates for storage for the technologies. Closes PR #32
</commit_message>
<xml_diff>
--- a/dac_offshore/clean_data/technologies_new/NewTechnologies.xlsx
+++ b/dac_offshore/clean_data/technologies_new/NewTechnologies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maiant/PycharmProjects/AdOpT-NET0_DAC-Offshore/dac_offshore/clean_data/technologies_new/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/8051917/PycharmProjects/AdOpT-NET0_DAC-Offshore/dac_offshore/clean_data/technologies_new/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B970953-C56B-E842-9483-313AFEB9052B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{840FCBE4-6471-B74F-8744-38094E7F9480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" xr2:uid="{64A87C74-33CB-4EAC-BDF2-6E9087B161C6}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15980" xr2:uid="{64A87C74-33CB-4EAC-BDF2-6E9087B161C6}"/>
   </bookViews>
   <sheets>
     <sheet name="NewTechnologies" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="105">
   <si>
     <t>offshore_new</t>
   </si>
@@ -330,15 +330,9 @@
     <t>NO_ST1</t>
   </si>
   <si>
-    <t>PermanentStorage_CO2_simple, DAC_Adsorption_offshore, HeatPump_SeaWaterSourced</t>
-  </si>
-  <si>
     <t>DAC_Adsorption_offshore, HeatPump_SeaWaterSourced</t>
   </si>
   <si>
-    <t>DAC_Adsorption_offshore, HeatPump_SeaWaterSourced, PermanentStorage_CO2_simple</t>
-  </si>
-  <si>
     <t>Offshore_DAC_only</t>
   </si>
   <si>
@@ -355,6 +349,12 @@
   </si>
   <si>
     <t>DAC_Adsorption_onshore, HeatPump_AirSourced_onshore</t>
+  </si>
+  <si>
+    <t>Offshore_Wind, Storage_Battery_Offshore, PermanentStorage_CO2_simple</t>
+  </si>
+  <si>
+    <t>Storage_Battery_Offshore, PermanentStorage_CO2_simple</t>
   </si>
 </sst>
 </file>
@@ -731,7 +731,9 @@
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="7" width="24" customWidth="1"/>
+    <col min="3" max="3" width="49.1640625" customWidth="1"/>
+    <col min="4" max="4" width="40.1640625" customWidth="1"/>
+    <col min="5" max="7" width="24" customWidth="1"/>
     <col min="8" max="8" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="13" width="15.33203125" customWidth="1"/>
     <col min="15" max="15" width="43" bestFit="1" customWidth="1"/>
@@ -751,13 +753,13 @@
         <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -765,10 +767,10 @@
         <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D2" t="s">
         <v>101</v>
+      </c>
+      <c r="C2" t="s">
+        <v>99</v>
       </c>
       <c r="E2" t="s">
         <v>96</v>
@@ -779,10 +781,10 @@
         <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D3" t="s">
         <v>101</v>
+      </c>
+      <c r="C3" t="s">
+        <v>99</v>
       </c>
       <c r="E3" t="s">
         <v>96</v>
@@ -793,10 +795,10 @@
         <v>94</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D4" t="s">
         <v>101</v>
+      </c>
+      <c r="C4" t="s">
+        <v>99</v>
       </c>
       <c r="E4" t="s">
         <v>96</v>
@@ -813,7 +815,7 @@
         <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -827,7 +829,7 @@
         <v>64</v>
       </c>
       <c r="E6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -841,7 +843,7 @@
         <v>64</v>
       </c>
       <c r="E7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -852,13 +854,10 @@
         <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -869,13 +868,10 @@
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -891,7 +887,7 @@
         <v>64</v>
       </c>
       <c r="E10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -902,13 +898,10 @@
         <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E11" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -919,13 +912,10 @@
         <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
-      </c>
-      <c r="D12" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -939,7 +929,7 @@
         <v>64</v>
       </c>
       <c r="E13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -952,13 +942,10 @@
         <v>0</v>
       </c>
       <c r="C14" t="s">
-        <v>64</v>
-      </c>
-      <c r="D14" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -972,7 +959,7 @@
         <v>64</v>
       </c>
       <c r="E15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -986,7 +973,7 @@
         <v>64</v>
       </c>
       <c r="E16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -1000,7 +987,7 @@
         <v>64</v>
       </c>
       <c r="E17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -1014,7 +1001,7 @@
         <v>64</v>
       </c>
       <c r="E18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1102,12 +1089,9 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>44</v>
-      </c>
-      <c r="D26" t="s">
-        <v>101</v>
-      </c>
-      <c r="E26" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E26" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1130,10 +1114,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E28" t="s">
         <v>96</v>
@@ -1147,10 +1128,7 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E29" t="s">
         <v>96</v>
@@ -1164,12 +1142,9 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>44</v>
-      </c>
-      <c r="D30" t="s">
-        <v>101</v>
-      </c>
-      <c r="E30" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E30" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1184,7 +1159,7 @@
         <v>44</v>
       </c>
       <c r="E31" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -1198,7 +1173,7 @@
         <v>44</v>
       </c>
       <c r="E32" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -1212,7 +1187,7 @@
         <v>44</v>
       </c>
       <c r="E33" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -1226,7 +1201,7 @@
         <v>44</v>
       </c>
       <c r="E34" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -1240,7 +1215,7 @@
         <v>44</v>
       </c>
       <c r="E35" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1254,7 +1229,7 @@
         <v>44</v>
       </c>
       <c r="E36" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1265,13 +1240,10 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>44</v>
-      </c>
-      <c r="D37" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E37" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1282,13 +1254,10 @@
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>44</v>
-      </c>
-      <c r="D38" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1302,7 +1271,7 @@
         <v>44</v>
       </c>
       <c r="E39" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -1313,13 +1282,10 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>44</v>
-      </c>
-      <c r="D40" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E40" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1333,7 +1299,7 @@
         <v>62</v>
       </c>
       <c r="D41" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -1347,7 +1313,7 @@
         <v>62</v>
       </c>
       <c r="D42" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -1361,7 +1327,7 @@
         <v>62</v>
       </c>
       <c r="D43" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -1375,7 +1341,7 @@
         <v>62</v>
       </c>
       <c r="D44" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1389,7 +1355,7 @@
         <v>62</v>
       </c>
       <c r="D45" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -1403,7 +1369,7 @@
         <v>62</v>
       </c>
       <c r="D46" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1417,7 +1383,7 @@
         <v>62</v>
       </c>
       <c r="D47" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1431,7 +1397,7 @@
         <v>62</v>
       </c>
       <c r="D48" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
@@ -1445,7 +1411,7 @@
         <v>62</v>
       </c>
       <c r="D49" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -1459,7 +1425,7 @@
         <v>62</v>
       </c>
       <c r="D50" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -1473,7 +1439,7 @@
         <v>62</v>
       </c>
       <c r="D51" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
@@ -1487,7 +1453,7 @@
         <v>62</v>
       </c>
       <c r="D52" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -1501,7 +1467,7 @@
         <v>62</v>
       </c>
       <c r="D53" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
@@ -1515,7 +1481,7 @@
         <v>62</v>
       </c>
       <c r="D54" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
@@ -1529,7 +1495,7 @@
         <v>62</v>
       </c>
       <c r="D55" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
@@ -1543,7 +1509,7 @@
         <v>62</v>
       </c>
       <c r="D56" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Include a new column in NewTechnologies.xlsx for CO2 Storage
</commit_message>
<xml_diff>
--- a/dac_offshore/clean_data/technologies_new/NewTechnologies.xlsx
+++ b/dac_offshore/clean_data/technologies_new/NewTechnologies.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/8051917/PycharmProjects/AdOpT-NET0_DAC-Offshore/dac_offshore/clean_data/technologies_new/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwiegner\PycharmProjects\AdOpT_DAC-Offshore\dac_offshore\clean_data\technologies_new\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{840FCBE4-6471-B74F-8744-38094E7F9480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1E4727-1253-4B73-BAD7-E91EAC044CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15980" xr2:uid="{64A87C74-33CB-4EAC-BDF2-6E9087B161C6}"/>
+    <workbookView xWindow="-21720" yWindow="-1965" windowWidth="21840" windowHeight="37920" xr2:uid="{64A87C74-33CB-4EAC-BDF2-6E9087B161C6}"/>
   </bookViews>
   <sheets>
     <sheet name="NewTechnologies" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">NewTechnologies!$A$1:$N$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">NewTechnologies!$A$1:$O$39</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="104">
   <si>
     <t>offshore_new</t>
   </si>
@@ -351,10 +351,7 @@
     <t>DAC_Adsorption_onshore, HeatPump_AirSourced_onshore</t>
   </si>
   <si>
-    <t>Offshore_Wind, Storage_Battery_Offshore, PermanentStorage_CO2_simple</t>
-  </si>
-  <si>
-    <t>Storage_Battery_Offshore, PermanentStorage_CO2_simple</t>
+    <t>CO2_Storage</t>
   </si>
 </sst>
 </file>
@@ -726,26 +723,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G60"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H60"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="49.1640625" customWidth="1"/>
-    <col min="4" max="4" width="40.1640625" customWidth="1"/>
-    <col min="5" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="13" width="15.33203125" customWidth="1"/>
-    <col min="15" max="15" width="43" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="34" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="43" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="25" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="24" customWidth="1"/>
-    <col min="22" max="22" width="15.33203125" customWidth="1"/>
-    <col min="24" max="24" width="43" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="49.140625" customWidth="1"/>
+    <col min="5" max="5" width="40.140625" customWidth="1"/>
+    <col min="6" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="14" width="15.28515625" customWidth="1"/>
+    <col min="16" max="16" width="43" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="34" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="43" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24" customWidth="1"/>
+    <col min="23" max="23" width="15.28515625" customWidth="1"/>
+    <col min="25" max="25" width="43" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -756,55 +753,58 @@
         <v>100</v>
       </c>
       <c r="D1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" t="s">
         <v>98</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>93</v>
       </c>
       <c r="B2" t="s">
         <v>101</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>99</v>
       </c>
-      <c r="E2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>95</v>
       </c>
       <c r="B3" t="s">
         <v>101</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>99</v>
       </c>
-      <c r="E3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>94</v>
       </c>
       <c r="B4" t="s">
         <v>101</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>99</v>
       </c>
-      <c r="E4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>61</v>
       </c>
@@ -814,11 +814,11 @@
       <c r="C5" t="s">
         <v>64</v>
       </c>
-      <c r="E5" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>60</v>
       </c>
@@ -828,11 +828,11 @@
       <c r="C6" t="s">
         <v>64</v>
       </c>
-      <c r="E6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>59</v>
       </c>
@@ -842,11 +842,11 @@
       <c r="C7" t="s">
         <v>64</v>
       </c>
-      <c r="E7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>58</v>
       </c>
@@ -854,13 +854,16 @@
         <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
-      </c>
-      <c r="E8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+      <c r="D8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>57</v>
       </c>
@@ -868,15 +871,18 @@
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>103</v>
-      </c>
-      <c r="E9" t="s">
-        <v>96</v>
-      </c>
-      <c r="F9" s="2"/>
+        <v>64</v>
+      </c>
+      <c r="D9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F9" t="s">
+        <v>96</v>
+      </c>
       <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>56</v>
       </c>
@@ -886,11 +892,11 @@
       <c r="C10" t="s">
         <v>64</v>
       </c>
-      <c r="E10" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>55</v>
       </c>
@@ -898,13 +904,16 @@
         <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
-      </c>
-      <c r="E11" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+      <c r="D11" t="s">
+        <v>99</v>
+      </c>
+      <c r="F11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -912,13 +921,16 @@
         <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
-      </c>
-      <c r="E12" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+      <c r="D12" t="s">
+        <v>99</v>
+      </c>
+      <c r="F12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>53</v>
       </c>
@@ -928,13 +940,13 @@
       <c r="C13" t="s">
         <v>64</v>
       </c>
-      <c r="E13" t="s">
-        <v>96</v>
-      </c>
-      <c r="F13" s="2"/>
+      <c r="F13" t="s">
+        <v>96</v>
+      </c>
       <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>52</v>
       </c>
@@ -942,13 +954,16 @@
         <v>0</v>
       </c>
       <c r="C14" t="s">
-        <v>103</v>
-      </c>
-      <c r="E14" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+      <c r="D14" t="s">
+        <v>99</v>
+      </c>
+      <c r="F14" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>51</v>
       </c>
@@ -958,11 +973,11 @@
       <c r="C15" t="s">
         <v>64</v>
       </c>
-      <c r="E15" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>50</v>
       </c>
@@ -972,11 +987,11 @@
       <c r="C16" t="s">
         <v>64</v>
       </c>
-      <c r="E16" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -986,11 +1001,11 @@
       <c r="C17" t="s">
         <v>64</v>
       </c>
-      <c r="E17" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -1000,11 +1015,11 @@
       <c r="C18" t="s">
         <v>64</v>
       </c>
-      <c r="E18" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F18" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -1015,7 +1030,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -1026,7 +1041,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1037,7 +1052,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -1048,7 +1063,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -1059,7 +1074,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -1070,7 +1085,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -1081,7 +1096,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>26</v>
       </c>
@@ -1089,13 +1104,16 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>104</v>
-      </c>
-      <c r="E26" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="D26" t="s">
+        <v>99</v>
+      </c>
+      <c r="F26" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -1106,7 +1124,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>37</v>
       </c>
@@ -1114,13 +1132,16 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>104</v>
-      </c>
-      <c r="E28" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="D28" t="s">
+        <v>99</v>
+      </c>
+      <c r="F28" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>38</v>
       </c>
@@ -1128,13 +1149,16 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
-      </c>
-      <c r="E29" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="D29" t="s">
+        <v>99</v>
+      </c>
+      <c r="F29" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>39</v>
       </c>
@@ -1142,13 +1166,16 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>104</v>
-      </c>
-      <c r="E30" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="D30" t="s">
+        <v>99</v>
+      </c>
+      <c r="F30" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>6</v>
       </c>
@@ -1158,11 +1185,11 @@
       <c r="C31" t="s">
         <v>44</v>
       </c>
-      <c r="E31" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F31" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>10</v>
       </c>
@@ -1172,11 +1199,11 @@
       <c r="C32" t="s">
         <v>44</v>
       </c>
-      <c r="E32" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F32" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -1186,11 +1213,11 @@
       <c r="C33" t="s">
         <v>44</v>
       </c>
-      <c r="E33" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F33" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>20</v>
       </c>
@@ -1200,11 +1227,11 @@
       <c r="C34" t="s">
         <v>44</v>
       </c>
-      <c r="E34" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -1214,11 +1241,11 @@
       <c r="C35" t="s">
         <v>44</v>
       </c>
-      <c r="E35" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F35" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>24</v>
       </c>
@@ -1228,11 +1255,11 @@
       <c r="C36" t="s">
         <v>44</v>
       </c>
-      <c r="E36" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F36" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>33</v>
       </c>
@@ -1240,13 +1267,16 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>104</v>
-      </c>
-      <c r="E37" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="D37" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>34</v>
       </c>
@@ -1254,13 +1284,16 @@
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>104</v>
-      </c>
-      <c r="E38" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="D38" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>35</v>
       </c>
@@ -1270,11 +1303,11 @@
       <c r="C39" t="s">
         <v>44</v>
       </c>
-      <c r="E39" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F39" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>36</v>
       </c>
@@ -1282,13 +1315,16 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>104</v>
-      </c>
-      <c r="E40" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="D40" t="s">
+        <v>99</v>
+      </c>
+      <c r="F40" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -1298,11 +1334,11 @@
       <c r="C41" t="s">
         <v>62</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>9</v>
       </c>
@@ -1312,11 +1348,11 @@
       <c r="C42" t="s">
         <v>62</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>16</v>
       </c>
@@ -1326,11 +1362,11 @@
       <c r="C43" t="s">
         <v>62</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>17</v>
       </c>
@@ -1340,11 +1376,11 @@
       <c r="C44" t="s">
         <v>62</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>18</v>
       </c>
@@ -1354,11 +1390,11 @@
       <c r="C45" t="s">
         <v>62</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>19</v>
       </c>
@@ -1368,11 +1404,11 @@
       <c r="C46" t="s">
         <v>62</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -1382,11 +1418,11 @@
       <c r="C47" t="s">
         <v>62</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>28</v>
       </c>
@@ -1396,11 +1432,11 @@
       <c r="C48" t="s">
         <v>62</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>29</v>
       </c>
@@ -1410,11 +1446,11 @@
       <c r="C49" t="s">
         <v>62</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>30</v>
       </c>
@@ -1424,11 +1460,11 @@
       <c r="C50" t="s">
         <v>62</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>31</v>
       </c>
@@ -1438,11 +1474,11 @@
       <c r="C51" t="s">
         <v>62</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>32</v>
       </c>
@@ -1452,11 +1488,11 @@
       <c r="C52" t="s">
         <v>62</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>40</v>
       </c>
@@ -1466,11 +1502,11 @@
       <c r="C53" t="s">
         <v>62</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>41</v>
       </c>
@@ -1480,11 +1516,11 @@
       <c r="C54" t="s">
         <v>62</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>42</v>
       </c>
@@ -1494,11 +1530,11 @@
       <c r="C55" t="s">
         <v>62</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>43</v>
       </c>
@@ -1508,36 +1544,39 @@
       <c r="C56" t="s">
         <v>62</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B58" s="1"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H58" s="2"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H59" s="2"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1553,13 +1592,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4641E15-13AD-4645-88BC-55D8D2E876ED}">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>63</v>
       </c>
@@ -1571,7 +1610,7 @@
         <v>'RE_only': 'RE only',</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>70</v>
       </c>
@@ -1583,7 +1622,7 @@
         <v>'Battery_on': 'Battery (onshore only)',</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -1595,7 +1634,7 @@
         <v>'Battery_off': 'Battery (offshore only)',</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1607,7 +1646,7 @@
         <v>'Battery_all': 'Battery (all)',</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>45</v>
       </c>
@@ -1619,7 +1658,7 @@
         <v>'ElectricityGrid_all': 'Grid Expansion (all)',</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>46</v>
       </c>
@@ -1631,7 +1670,7 @@
         <v>'Hydrogen_Baseline': 'Hydrogen (all)',</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>72</v>
       </c>
@@ -1643,7 +1682,7 @@
         <v>'Hydrogen_H1': 'Hydrogen (no storage)',</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>73</v>
       </c>
@@ -1655,7 +1694,7 @@
         <v>'Hydrogen_H2': 'Hydrogen (no hydrogen offshore)',</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>74</v>
       </c>
@@ -1667,7 +1706,7 @@
         <v>'Hydrogen_H3': 'Hydrogen (no hydrogen onshore)',</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>75</v>
       </c>
@@ -1679,7 +1718,7 @@
         <v>'Hydrogen_H4': 'Hydrogen (local use only)',</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>47</v>
       </c>
@@ -1691,7 +1730,7 @@
         <v>'All': 'All Pathways',</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>66</v>
       </c>
@@ -1704,7 +1743,7 @@
         <v>'RE_only_no_onshore_wind': 'RE only - no onshore wind',</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>76</v>
       </c>
@@ -1717,7 +1756,7 @@
         <v>'Battery_on_no_onshore_wind': 'Battery (onshore only) - no onshore wind',</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -1730,7 +1769,7 @@
         <v>'Battery_off_no_onshore_wind': 'Battery (offshore only) - no onshore wind',</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -1743,7 +1782,7 @@
         <v>'Battery_all_no_onshore_wind': 'Battery (all) - no onshore wind',</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>68</v>
       </c>
@@ -1756,7 +1795,7 @@
         <v>'ElectricityGrid_all_no_onshore_wind': 'Grid Expansion (all) - no onshore wind',</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>69</v>
       </c>
@@ -1769,7 +1808,7 @@
         <v>'Hydrogen_Baseline_no_onshore_wind': 'Hydrogen (all) - no onshore wind',</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>78</v>
       </c>
@@ -1782,7 +1821,7 @@
         <v>'Hydrogen_H1_no_onshore_wind': 'Hydrogen (no storage) - no onshore wind',</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>79</v>
       </c>
@@ -1795,7 +1834,7 @@
         <v>'Hydrogen_H2_no_onshore_wind': 'Hydrogen (no hydrogen offshore) - no onshore wind',</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>80</v>
       </c>
@@ -1808,7 +1847,7 @@
         <v>'Hydrogen_H3_no_onshore_wind': 'Hydrogen (no hydrogen onshore) - no onshore wind',</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>81</v>
       </c>
@@ -1821,7 +1860,7 @@
         <v>'Hydrogen_H4_no_onshore_wind': 'Hydrogen (local use only) - no onshore wind',</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>65</v>
       </c>

</xml_diff>